<commit_message>
docs v1.8.1: RF-004f cierre al cerrar navegador, ADR-17 enmendado, US-045, REPORTE_7 (F-27, T-17..T-19)
</commit_message>
<xml_diff>
--- a/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
+++ b/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
@@ -480,7 +480,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REPORTE 7 — Entrega definitiva v1.8.0 (18/10/2026)</t>
+          <t>REPORTE 7 — Entrega definitiva v1.8.1 (18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>1.8.0</t>
+          <t>1.8.1</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>v1.8.0 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
+          <t>v1.8.1 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Recorrido por roles + panel Agente IA (apagado por defecto) + sesión única entre pestañas</t>
+          <t>Recorrido por roles + panel Agente IA (apagado por defecto) + sesión única entre pestañas + cierre de sesión al cerrar el navegador</t>
         </is>
       </c>
     </row>
@@ -910,7 +910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2005,6 +2005,46 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>F-27</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Cierre de sesión al cerrar el navegador (v1.8.1)</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Obligatoria</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Terminada y probada</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Heartbeat por pestaña; cierre detectado al reabrir; F5 conserva sesión</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>navegador local</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2016,7 +2056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2829,6 +2869,147 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>T-17</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>F-27</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Cerrar todas las pestañas y reabrir la app</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Login + aviso "Se cerró la sesión" + refresh 200/logout 204 en servidor</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Pasada</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>navegador local</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>T-18</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>F-27</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Recarga (F5) con sesión abierta</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Conserva la sesión (navigation.type=reload)</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Pasada</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>navegador local</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>T-19</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>F-27</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Pestaña nueva con otra pestaña viva + cierre de una sola</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Hereda sesión sin logout; la restante sigue activa</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Pasada</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>navegador local</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix Seguridad v1.8.2: restablecimiento de contrasena sin enumerar usuarios (respuesta generica siempre + envio via Celery)
</commit_message>
<xml_diff>
--- a/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
+++ b/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
@@ -480,7 +480,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REPORTE 7 — Entrega definitiva v1.8.1 (18/10/2026)</t>
+          <t>REPORTE 7 — Entrega definitiva v1.8.2 (18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>1.8.1</t>
+          <t>1.8.2</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>v1.8.1 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
+          <t>v1.8.2 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
         </is>
       </c>
     </row>
@@ -2056,7 +2056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3010,6 +3010,53 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>T-20</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>F-01</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Restablecimiento con correo inexistente / existente / desactivado</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Siempre 200 con el mismo mensaje genérico (sin enumerar); el correo sale por Celery sin demorar la respuesta</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Pasada</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>navegador local + worker</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v1.8.4: alcance de datos por rol (RF-004g) - /groups/ y /teams/ acotados al grupo del usuario (admin: catalogo completo, detalle ajeno 404) - /dashboard/ solo ADMIN/SUPERVISOR/SOPORTE: DESPACHADOR recibe 403 y el front deja de pedirlo - suite 40/40 (CatalogVisibilityTests + DashboardAccessTests) - docs: RF-004g, US-046, REPORTE_7 F-28/T-21..T-23, build verde
</commit_message>
<xml_diff>
--- a/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
+++ b/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
@@ -480,7 +480,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REPORTE 7 — Entrega definitiva v1.8.2 (18/10/2026)</t>
+          <t>REPORTE 7 — Entrega definitiva v1.8.4 (18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>1.8.2</t>
+          <t>1.8.4</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>v1.8.2 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
+          <t>v1.8.4 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.0 (ramas main/dev)</t>
+          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.4 (ramas main/dev)</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Recorrido por roles + panel Agente IA (apagado por defecto) + sesión única entre pestañas + cierre de sesión al cerrar el navegador</t>
+          <t>Recorrido por roles + panel Agente IA (apagado por defecto) + sesión única entre pestañas + cierre de sesión al cerrar el navegador + datos acotados por rol</t>
         </is>
       </c>
     </row>
@@ -910,7 +910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2045,6 +2045,46 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>F-28</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Alcance de datos por rol: catálogos acotados y dashboard por perfil (v1.8.4)</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Obligatoria</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Terminada y probada</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>/groups/ y /teams/ solo del grupo del usuario; /dashboard/ 403 para DESPACHADOR; suite 40/40</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>API + navegador</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2056,7 +2096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2746,12 +2786,12 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Suite backend completa v1.8.0</t>
+          <t>Suite backend completa (v1.8.4)</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>30/30 OK</t>
+          <t>40/40 OK</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -3052,6 +3092,147 @@
         </is>
       </c>
       <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>T-21</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>F-28</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Token de DESPACHADOR contra /groups/, /teams/ y detalle de grupo/equipo ajeno</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Solo catálogo propio ('tigo'); detalle ajeno 404; el admin conserva los 7 grupos y 8 equipos</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Pasada</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>API local</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>T-22</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>F-28</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>GET /dashboard/ con token de DESPACHADOR</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>403 "Tu perfil no tiene acceso al panel de resumen"; ADMIN/SUPERVISOR/SOPORTE responden 200</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Pasada</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>manage.py test</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>T-23</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>F-28</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Navegación del despacho tras el cambio (red y pantallas)</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Sin llamada a dashboard/; grupos y equipos solo 'tigo'; Tickets/Validaciones/Escalados y modal Nuevo ticket operativos; admin sin cambios</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Pasada</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>navegador local</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
         <is>
           <t>18/10/2026</t>
         </is>

</xml_diff>

<commit_message>
v1.8.5: bandeja ordenada por prioridad por defecto - sort inicial 'prioridad' en TicketsView (antes 'recientes'); selector conserva recientes/antiguos - docs: RF-008/009/010 marca orden por defecto; RF-039/040/US-039 delimina modos de la IA (automatico o sugerencia, configurable) - REPORTE_7 v1.8.5 con fila T-24 - docx regenerado, build verde
</commit_message>
<xml_diff>
--- a/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
+++ b/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
@@ -480,7 +480,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REPORTE 7 — Entrega definitiva v1.8.4 (18/10/2026)</t>
+          <t>REPORTE 7 — Entrega definitiva v1.8.5 (18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>1.8.4</t>
+          <t>1.8.5</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>v1.8.4 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
+          <t>v1.8.5 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.4 (ramas main/dev)</t>
+          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.5 (ramas main/dev)</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Apagado por defecto; solo sugiere bajo umbral</t>
+          <t>Apagado por defecto; encendido decide el admin: aplica sola (umbral, servicios, allow_lower, cooldown 24h) o solo sugiere</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -2096,7 +2096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3238,6 +3238,53 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>T-24</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>F-06</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Bandeja de tickets con orden por defecto 'prioridad' (v1.8.5)</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Crítica→Alta→Media→Baja, más antiguas primero a igual prioridad; el selector sigue ofreciendo recientes/antiguos</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Pasada</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>navegador local</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v1.8.6 (docs): ingenieria inversa y REPORTE_7 reflejan orden estado+prioridad con cerrados al fondo
</commit_message>
<xml_diff>
--- a/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
+++ b/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
@@ -480,7 +480,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REPORTE 7 — Entrega definitiva v1.8.5 (18/10/2026)</t>
+          <t>REPORTE 7 — Entrega definitiva v1.8.6 (18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>1.8.5</t>
+          <t>1.8.6</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>v1.8.5 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
+          <t>v1.8.6 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.5 (ramas main/dev)</t>
+          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.6 (ramas main/dev)</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3285,6 +3285,53 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>T-25</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>F-06</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Bandeja ordena por estado + prioridad, cerrados al fondo (v1.8.6)</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Cerrados SIEMPRE al fondo; dentro de cada estado (Abierto/Asignado/En proceso/Escalado/Validación) prioridad Crítica→Alta→Media→Baja; a igual estado y prioridad, las más antiguas</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Pasada</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>navegador local</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v1.8.7: Ollama como servicio del stack de produccion (compose.prod + runbook §6)
</commit_message>
<xml_diff>
--- a/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
+++ b/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
@@ -480,7 +480,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REPORTE 7 — Entrega definitiva v1.8.6 (18/10/2026)</t>
+          <t>REPORTE 7 — Entrega definitiva v1.8.7 (18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>1.8.6</t>
+          <t>1.8.7</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>v1.8.6 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
+          <t>v1.8.7 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.6 (ramas main/dev)</t>
+          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.7 (ramas main/dev)</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3332,6 +3332,53 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>T-26</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>F-25</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Despliegue</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Ollama como servicio del stack de producción (v1.8.7)</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Servicio 'ollama' con volumen ollama_models y puerto 11434 NO publicado; api/worker apuntan a http://ollama:11434 por red interna; env IA_VISION_ENABLED/IA_AUTO_APPLY parametrizados por .env; docker compose -f compose.prod.yaml config válido</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Pasada</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>docker compose config + Runbook §6</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v1.8.8: agente IA ~3x mas rapido (think:false + espera 60->20s + keep_alive 30m)
</commit_message>
<xml_diff>
--- a/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
+++ b/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
@@ -480,7 +480,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REPORTE 7 — Entrega definitiva v1.8.7 (18/10/2026)</t>
+          <t>REPORTE 7 — Entrega definitiva v1.8.8 (18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>1.8.7</t>
+          <t>1.8.8</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>v1.8.7 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
+          <t>v1.8.8 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.7 (ramas main/dev)</t>
+          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.8 (ramas main/dev)</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3379,6 +3379,53 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>T-27</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>F-20</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Optimización de tiempos del agente IA (v1.8.8), medición con imagen y prompts reales</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Revisor con think:false: qwen3:4b de 54 s a 7 s yéndose directo al JSON; espera entre etapas 60→20 s; OLLAMA_KEEP_ALIVE=30m en compose. Análisis completo ~2 min → ~40-60 s. moondream descartado (20 s y salida vacía en CPU). Suite 40/40 OK</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>Pasada</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>bench local Ollama + imagen real del ticket + suite</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v1.8.9: bandeja paginada (25 por pagina) y ventana de 30 dias en el listado (RF-043)
</commit_message>
<xml_diff>
--- a/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
+++ b/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
@@ -480,7 +480,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REPORTE 7 — Entrega definitiva v1.8.8 (18/10/2026)</t>
+          <t>REPORTE 7 — Entrega definitiva v1.8.9 (18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>1.8.8</t>
+          <t>1.8.9</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>v1.8.8 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
+          <t>v1.8.9 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.8 (ramas main/dev)</t>
+          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.9 (ramas main/dev)</t>
         </is>
       </c>
     </row>
@@ -910,7 +910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2085,6 +2085,46 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>F-29</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Tickets</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Bandeja paginada (25 por página) y ventana de 30 días en el listado (v1.8.9)</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Obligatoria</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Terminada y probada</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>Paginador UI sobre la lista ordenada por estado+prioridad; API acotada por defecto (no cerrados + cerrados de 30 días, ?todo=1 para histórico)</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>manage.py test + navegador</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2096,7 +2136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3426,6 +3466,53 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>T-28</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>F-29</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Bandeja paginada y con ventana por defecto en el listado (v1.8.9, RF-043)</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>63 tickets → paginador '63 tickets · Página 1 de 3' con 25 filas; 'Siguiente' carga la página 2 (filas distintas) y habilita 'Anterior'; API por defecto excluye cerrados &gt;30 días (63 vs 69 con ?todo=1) sin tocar los no cerrados; orden global estado+prioridad intacto. Suite 42/42 OK</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Pasada</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>manage.py test + navegador</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v1.8.10: mostrar/ocultar contrasena (boton de ojo) en los 5 campos de clave (RF-044)
</commit_message>
<xml_diff>
--- a/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
+++ b/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
@@ -480,7 +480,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REPORTE 7 — Entrega definitiva v1.8.9 (18/10/2026)</t>
+          <t>REPORTE 7 — Entrega definitiva v1.8.10 (18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>1.8.9</t>
+          <t>1.8.10</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>v1.8.9 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
+          <t>v1.8.10 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.9 (ramas main/dev)</t>
+          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.10 (ramas main/dev)</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3513,6 +3513,53 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>T-29</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>F-10</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Botón mostrar/ocultar contraseña en los campos de clave (v1.8.10, RF-044)</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Login: al escribir 'Prueba1234!' el campo es type=password; el ojo lo cambia a type=text conservando el valor y la etiqueta accesible pasa a 'Ocultar contraseña'; el segundo clic regresa a password. Aplica en los 5 campos de clave (login, restablecimiento por enlace, modal de usuario y restablecimiento por admin)</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Pasada</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>navegador local</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v1.8.11: cuentas blindadas - edicion de usuario sin contrasena y correo/restablecimiento solo admin (RF-045)
</commit_message>
<xml_diff>
--- a/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
+++ b/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
@@ -480,7 +480,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REPORTE 7 — Entrega definitiva v1.8.10 (18/10/2026)</t>
+          <t>REPORTE 7 — Entrega definitiva v1.8.11 (18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>1.8.10</t>
+          <t>1.8.11</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>v1.8.10 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
+          <t>v1.8.11 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.10 (ramas main/dev)</t>
+          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.11 (ramas main/dev)</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3560,6 +3560,53 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>T-30</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>F-23</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Cuentas blindadas: edición sin contraseña y correo/restablecimiento solo admin (v1.8.11, RF-045)</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Supervisor: PATCH {password} en /users/{id} → 400 y la clave no cambia; PATCH {email} distinto → 400; con el correo sin cambios la edición normal sigue 200. Admin: restablecer contraseña sigue 200. UI verificada en navegador como admin (edición sin campo de contraseña, correo editable, botón «Contraseña» visible) y como supervisor (sin botón «Contraseña», correo de solo lectura). Suite 45/45 OK</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Pasada</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>manage.py test + navegador</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v1.8.12: quita el aviso de texto del modal de edicion de usuarios (redundante, RF-045)
</commit_message>
<xml_diff>
--- a/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
+++ b/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
@@ -480,7 +480,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REPORTE 7 — Entrega definitiva v1.8.11 (18/10/2026)</t>
+          <t>REPORTE 7 — Entrega definitiva v1.8.12 (18/10/2026)</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>1.8.11</t>
+          <t>1.8.12</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>v1.8.11 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
+          <t>v1.8.12 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.11 (ramas main/dev)</t>
+          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.12 (ramas main/dev)</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3607,6 +3607,53 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>T-31</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>F-23</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Se elimina el aviso de texto del modal de edición (v1.8.12)</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>El modal 'Editar usuario' ya no muestra el párrafo 'La contraseña no se cambia en la edición...' (redundante: el formulario no ofrece contraseña y el botón «Contraseña» es solo de admin); el resto del formulario (nombre, correo, equipos, activo) queda igual. Verificado en navegador como admin y como supervisor</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Pasada</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>navegador local</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v1.8.13: build del frontend en Node 24 LTS (v24.22.1, fixes de seguridad 20/10/2026); node 20 estaba en EOL
</commit_message>
<xml_diff>
--- a/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
+++ b/Evidencias y Documentacion/REPORTE_7_Entrega_Definitiva.xlsx
@@ -480,7 +480,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REPORTE 7 — Entrega definitiva v1.8.12 (18/10/2026)</t>
+          <t>REPORTE 7 — Entrega definitiva v1.8.13 (23/10/2026)</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>1.8.12</t>
+          <t>1.8.13</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>18/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>v1.8.12 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
+          <t>v1.8.13 — server local Ubuntu (IP fija interna, externo vía VPN)</t>
         </is>
       </c>
     </row>
@@ -765,7 +765,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Docker, PostgreSQL 16, Redis 7, Python 3.13, Node 20, Daphne, Celery, Tesseract</t>
+          <t>Docker, PostgreSQL 16, Redis 7, Python 3.13, Node 24 (build del frontend), Daphne, Celery, Tesseract</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.12 (ramas main/dev)</t>
+          <t>GitHub GabrielSazo/Soporte-Despacho, tag v1.8.13 (ramas main/dev)</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3654,6 +3654,53 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>T-32</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>F-25</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Despliegue</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Build del frontend en Node 24 LTS — fixes de seguridad del 20/10/2026 (v1.8.13)</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Etapa de build del Dockerfile.frontend y servicio dev pasan de node:20-alpine (EOL abril 2026) a node:24-alpine = v24.22.1 (LTS Krypton; el release de seguridad del 20/10/2026 también trajo 22.23.4 y 26.12.1 en las demás líneas activas, verificado en nodejs.org/dist). Imagen de frontend reconstruida completa con la nueva base: mismos hashes de assets (index-Bez9QnLE.js) y nginx final sin Node</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Pasada</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>docker build local + nodejs.org</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>